<commit_message>
Add TESTCD_NCIt column: make DSS-level NCIt codes visible when they differ from BC-level NCIt_Code (~7 cases). New QC-14 check. Diagnostic notebook included.
</commit_message>
<xml_diff>
--- a/cosmos-bc-dss/reports/COSMoS_BC_DSS_QC.xlsx
+++ b/cosmos-bc-dss/reports/COSMoS_BC_DSS_QC.xlsx
@@ -11,7 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="QC_Report" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'QC_Report'!$A$1:$E$16</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'QC_Report'!$A$1:$E$17</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -756,7 +756,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E16"/>
+  <dimension ref="A1:E17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -1160,8 +1160,33 @@
         </is>
       </c>
     </row>
+    <row r="17">
+      <c r="A17" s="11" t="inlineStr">
+        <is>
+          <t>QC-14</t>
+        </is>
+      </c>
+      <c r="B17" s="12" t="inlineStr">
+        <is>
+          <t>INFO</t>
+        </is>
+      </c>
+      <c r="C17" s="11" t="inlineStr">
+        <is>
+          <t>TESTCD_NCIt differs from NCIt_Code</t>
+        </is>
+      </c>
+      <c r="D17" s="11" t="n">
+        <v>7</v>
+      </c>
+      <c r="E17" s="11" t="inlineStr">
+        <is>
+          <t>HEIGHT (Body Height): BC=C164634 TESTCD=C25347 | WEIGHT (Body Weight): BC=C81328 TESTCD=C25208 | INTP (Electrocardiogram Analysis): BC=C181655 TESTCD=C41255 | GLUCPE (Glucose Measurement): BC=C105585 TESTCD=C163446 | MICROCY (Microcyte to Erythrocyte Ratio): BC=C201227 TESTCD=C64822 | LENGTH (Organ Craniocaudal Length Meas): BC=C135509 TESTCD=C25334 | HCG (Serum HCG Measurement): BC=C73495 TESTCD=C64851</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:E16"/>
+  <autoFilter ref="A1:E17"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Add BC_Scope (Subject/Study) column, QC-15 for study-level BCs. Add TESTCD_NCIt column, QC-14 for BC/TESTCD NCIt mismatches. Update all docs.
</commit_message>
<xml_diff>
--- a/cosmos-bc-dss/reports/COSMoS_BC_DSS_QC.xlsx
+++ b/cosmos-bc-dss/reports/COSMoS_BC_DSS_QC.xlsx
@@ -11,7 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="QC_Report" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'QC_Report'!$A$1:$E$17</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'QC_Report'!$A$1:$E$18</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -756,7 +756,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E17"/>
+  <dimension ref="A1:E18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -1185,8 +1185,33 @@
         </is>
       </c>
     </row>
+    <row r="18">
+      <c r="A18" s="11" t="inlineStr">
+        <is>
+          <t>QC-15</t>
+        </is>
+      </c>
+      <c r="B18" s="12" t="inlineStr">
+        <is>
+          <t>INFO</t>
+        </is>
+      </c>
+      <c r="C18" s="11" t="inlineStr">
+        <is>
+          <t>BC_Scope=Study: trial-level metadata included as BCs</t>
+        </is>
+      </c>
+      <c r="D18" s="11" t="n">
+        <v>193</v>
+      </c>
+      <c r="E18" s="11" t="inlineStr">
+        <is>
+          <t>192 BCs, 129 DSS rows, 63 hierarchy rows | Domains: TS</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:E17"/>
+  <autoFilter ref="A1:E18"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
updated the flatten to handle more code lists for method and specimen
</commit_message>
<xml_diff>
--- a/cosmos-bc-dss/reports/COSMoS_BC_DSS_QC.xlsx
+++ b/cosmos-bc-dss/reports/COSMoS_BC_DSS_QC.xlsx
@@ -20,7 +20,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="7">
+  <fonts count="6">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -36,21 +36,17 @@
       <b val="1"/>
     </font>
     <font>
-      <b val="1"/>
-      <color rgb="009C0006"/>
+      <color rgb="00276221"/>
     </font>
     <font>
       <b val="1"/>
       <color rgb="009C6500"/>
     </font>
     <font>
-      <color rgb="00276221"/>
-    </font>
-    <font>
       <color rgb="007B6000"/>
     </font>
   </fonts>
-  <fills count="8">
+  <fills count="7">
     <fill>
       <patternFill/>
     </fill>
@@ -71,20 +67,14 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FFC7CE"/>
-        <bgColor rgb="00FFC7CE"/>
+        <fgColor rgb="00C6EFCE"/>
+        <bgColor rgb="00C6EFCE"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00FFEB9C"/>
         <bgColor rgb="00FFEB9C"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00C6EFCE"/>
-        <bgColor rgb="00C6EFCE"/>
       </patternFill>
     </fill>
     <fill>
@@ -120,7 +110,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
@@ -147,12 +137,6 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -577,7 +561,7 @@
       <c r="B5" s="2" t="inlineStr"/>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>Generated: 2026-04-09</t>
+          <t>Generated: 2026-04-16</t>
         </is>
       </c>
     </row>
@@ -792,7 +776,7 @@
       </c>
       <c r="B2" s="5" t="inlineStr">
         <is>
-          <t>ERROR</t>
+          <t>PASS</t>
         </is>
       </c>
       <c r="C2" s="4" t="inlineStr">
@@ -801,13 +785,9 @@
         </is>
       </c>
       <c r="D2" s="4" t="n">
-        <v>4</v>
-      </c>
-      <c r="E2" s="4" t="inlineStr">
-        <is>
-          <t>C113243 (2 usages) | C449 (26 usages) | C812 (7 usages) | C95940 (3 usages)</t>
-        </is>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="E2" s="4" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" s="6" t="inlineStr">
@@ -826,84 +806,80 @@
         </is>
       </c>
       <c r="D3" s="6" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E3" s="6" t="inlineStr">
         <is>
-          <t>AUTOPSY (1 usages) | C179788 (1 usages) | PINCH DYNAMOMETRY (1 usages)</t>
+          <t>AUTOPSY (1 usages) | PINCH DYNAMOMETRY (1 usages)</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="8" t="inlineStr">
+      <c r="A4" s="4" t="inlineStr">
         <is>
           <t>QC-03</t>
         </is>
       </c>
-      <c r="B4" s="9" t="inlineStr">
+      <c r="B4" s="5" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
       </c>
-      <c r="C4" s="8" t="inlineStr">
+      <c r="C4" s="4" t="inlineStr">
         <is>
           <t>CT unmapped: Unit</t>
         </is>
       </c>
-      <c r="D4" s="8" t="n">
+      <c r="D4" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="E4" s="8" t="inlineStr"/>
+      <c r="E4" s="4" t="inlineStr"/>
     </row>
     <row r="5">
-      <c r="A5" s="10" t="inlineStr">
+      <c r="A5" s="8" t="inlineStr">
         <is>
           <t>QC-04</t>
         </is>
       </c>
-      <c r="B5" s="11" t="inlineStr">
+      <c r="B5" s="9" t="inlineStr">
         <is>
           <t>INFO</t>
         </is>
       </c>
-      <c r="C5" s="10" t="inlineStr">
+      <c r="C5" s="8" t="inlineStr">
         <is>
           <t>DSS rows with no TESTCD (no CT test code in COSMoS source)</t>
         </is>
       </c>
-      <c r="D5" s="10" t="n">
+      <c r="D5" s="8" t="n">
         <v>48</v>
       </c>
-      <c r="E5" s="10" t="inlineStr">
+      <c r="E5" s="8" t="inlineStr">
         <is>
           <t>ADVEVENT (DS) | ARIGEABCH (IS) | ARIGEABFP (IS) | ARIGEABM (IS) | ARIGEABMR (IS) | ARIGEABPC (IS) | BRTHDTC (DM) | PROTCOMP (DS) | CTSCAN (PR) | CTSCANCHEST (PR)</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="6" t="inlineStr">
+      <c r="A6" s="4" t="inlineStr">
         <is>
           <t>QC-05</t>
         </is>
       </c>
-      <c r="B6" s="7" t="inlineStr">
-        <is>
-          <t>WARNING</t>
-        </is>
-      </c>
-      <c r="C6" s="6" t="inlineStr">
+      <c r="B6" s="5" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="C6" s="4" t="inlineStr">
         <is>
           <t>Specimen present but Specimen_NCIt blank</t>
         </is>
       </c>
-      <c r="D6" s="6" t="n">
-        <v>38</v>
-      </c>
-      <c r="E6" s="6" t="inlineStr">
-        <is>
-          <t>C449 | C812 | C113243 | C95940</t>
-        </is>
-      </c>
+      <c r="D6" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="E6" s="4" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" s="6" t="inlineStr">
@@ -956,50 +932,50 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="10" t="inlineStr">
+      <c r="A9" s="8" t="inlineStr">
         <is>
           <t>QC-08</t>
         </is>
       </c>
-      <c r="B9" s="11" t="inlineStr">
+      <c r="B9" s="9" t="inlineStr">
         <is>
           <t>INFO</t>
         </is>
       </c>
-      <c r="C9" s="10" t="inlineStr">
+      <c r="C9" s="8" t="inlineStr">
         <is>
           <t>Multi-result DSS (same TESTCD+Domain+Specimen)</t>
         </is>
       </c>
-      <c r="D9" s="10" t="n">
+      <c r="D9" s="8" t="n">
         <v>32</v>
       </c>
-      <c r="E9" s="10" t="inlineStr">
-        <is>
-          <t>IS ARIGEAB (SERUM; SERUM OR PLASMA; BLOOD) x87 | IS MBIGGAB (SERUM; SERUM OR PLASMA; BLOOD) x63 | IS ARIGGAB (SERUM; SERUM OR PLASMA; BLOOD) x53 | IS MBIMAB (SERUM; SERUM OR PLASMA; BLOOD) x52 | IS ARIGAAB (SERUM; SERUM OR PLASMA; BLOOD) x17 | IS ATIGMAB (SERUM; SERUM OR PLASMA; BLOOD) x12 | GF SEQREAR (C449) x6 | GF SNV (C449) x6 | GF SHRTVAR (C449) x5 | GF TRNSCPTN (C812) x5</t>
+      <c r="E9" s="8" t="inlineStr">
+        <is>
+          <t>IS ARIGEAB (SERUM; SERUM OR PLASMA; BLOOD) x87 | IS MBIGGAB (SERUM; SERUM OR PLASMA; BLOOD) x63 | IS ARIGGAB (SERUM; SERUM OR PLASMA; BLOOD) x53 | IS MBIMAB (SERUM; SERUM OR PLASMA; BLOOD) x52 | IS ARIGAAB (SERUM; SERUM OR PLASMA; BLOOD) x17 | IS ATIGMAB (SERUM; SERUM OR PLASMA; BLOOD) x12 | GF SEQREAR (DNA) x6 | GF SNV (DNA) x6 | GF SHRTVAR (DNA) x5 | GF TRNSCPTN (RNA) x5</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="10" t="inlineStr">
+      <c r="A10" s="8" t="inlineStr">
         <is>
           <t>QC-09</t>
         </is>
       </c>
-      <c r="B10" s="11" t="inlineStr">
+      <c r="B10" s="9" t="inlineStr">
         <is>
           <t>INFO</t>
         </is>
       </c>
-      <c r="C10" s="10" t="inlineStr">
+      <c r="C10" s="8" t="inlineStr">
         <is>
           <t>BC_only_no_DS (192 BCs) -- top categories</t>
         </is>
       </c>
-      <c r="D10" s="10" t="n">
+      <c r="D10" s="8" t="n">
         <v>192</v>
       </c>
-      <c r="E10" s="10" t="inlineStr">
+      <c r="E10" s="8" t="inlineStr">
         <is>
           <t>QRS: 119 | Functional Assessment: 96 | ADAS-Cog: 95 | ADC: 95 | Alzheimer's Disease Assessment Scale-Cognitive CDISC Version Functional Test: 95 | ADAS-Cog CDISC Version Functional Test Question: 94 | Laboratory Tests: 16 | Clinical or Research Assessment Classification: 14 | Gene Expression Analysis: 11 | Genetic Testing: 10</t>
         </is>
@@ -1081,46 +1057,46 @@
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="8" t="inlineStr">
+      <c r="A14" s="4" t="inlineStr">
         <is>
           <t>QC-11c</t>
         </is>
       </c>
-      <c r="B14" s="9" t="inlineStr">
+      <c r="B14" s="5" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
       </c>
-      <c r="C14" s="8" t="inlineStr">
+      <c r="C14" s="4" t="inlineStr">
         <is>
           <t>Result_Scale: no unexpected values</t>
         </is>
       </c>
-      <c r="D14" s="8" t="n">
+      <c r="D14" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="E14" s="8" t="inlineStr"/>
+      <c r="E14" s="4" t="inlineStr"/>
     </row>
     <row r="15">
-      <c r="A15" s="10" t="inlineStr">
+      <c r="A15" s="8" t="inlineStr">
         <is>
           <t>QC-12</t>
         </is>
       </c>
-      <c r="B15" s="11" t="inlineStr">
+      <c r="B15" s="9" t="inlineStr">
         <is>
           <t>INFO</t>
         </is>
       </c>
-      <c r="C15" s="10" t="inlineStr">
+      <c r="C15" s="8" t="inlineStr">
         <is>
           <t>Placeholder BC_IDs (NCIt code pending)</t>
         </is>
       </c>
-      <c r="D15" s="10" t="n">
+      <c r="D15" s="8" t="n">
         <v>6</v>
       </c>
-      <c r="E15" s="10" t="inlineStr">
+      <c r="E15" s="8" t="inlineStr">
         <is>
           <t>NEW_LZZT (TTS Acceptability Survey) | NEW_LZZT4 (TTS Acceptability Survey -  Pa) | NEW_LZZT1 (TTS Acceptability Survey -  Pa) | NEW_LZZT3 (TTS Acceptability Survey -  Pa) | NEW_LZZT2 (TTS Acceptability Survey -  Pa) | NEW_1 (Urine Glucose Test Strip Measu)</t>
         </is>
@@ -1152,50 +1128,50 @@
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="10" t="inlineStr">
+      <c r="A17" s="8" t="inlineStr">
         <is>
           <t>QC-14</t>
         </is>
       </c>
-      <c r="B17" s="11" t="inlineStr">
+      <c r="B17" s="9" t="inlineStr">
         <is>
           <t>INFO</t>
         </is>
       </c>
-      <c r="C17" s="10" t="inlineStr">
+      <c r="C17" s="8" t="inlineStr">
         <is>
           <t>TESTCD_NCIt differs from NCIt_Code</t>
         </is>
       </c>
-      <c r="D17" s="10" t="n">
+      <c r="D17" s="8" t="n">
         <v>7</v>
       </c>
-      <c r="E17" s="10" t="inlineStr">
+      <c r="E17" s="8" t="inlineStr">
         <is>
           <t>HEIGHT (Body Height): BC=C164634 TESTCD=C25347 | WEIGHT (Body Weight): BC=C81328 TESTCD=C25208 | INTP (Electrocardiogram Analysis): BC=C181655 TESTCD=C41255 | GLUCPE (Glucose Measurement): BC=C105585 TESTCD=C163446 | MICROCY (Microcyte to Erythrocyte Ratio): BC=C201227 TESTCD=C64822 | LENGTH (Organ Craniocaudal Length Meas): BC=C135509 TESTCD=C25334 | HCG (Serum HCG Measurement): BC=C73495 TESTCD=C64851</t>
         </is>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="10" t="inlineStr">
+      <c r="A18" s="8" t="inlineStr">
         <is>
           <t>QC-15</t>
         </is>
       </c>
-      <c r="B18" s="11" t="inlineStr">
+      <c r="B18" s="9" t="inlineStr">
         <is>
           <t>INFO</t>
         </is>
       </c>
-      <c r="C18" s="10" t="inlineStr">
+      <c r="C18" s="8" t="inlineStr">
         <is>
           <t>BC_Scope=Study: trial-level metadata included as BCs</t>
         </is>
       </c>
-      <c r="D18" s="10" t="n">
+      <c r="D18" s="8" t="n">
         <v>193</v>
       </c>
-      <c r="E18" s="10" t="inlineStr">
+      <c r="E18" s="8" t="inlineStr">
         <is>
           <t>192 BCs, 129 DSS rows, 63 hierarchy rows | Domains: TS</t>
         </is>

</xml_diff>